<commit_message>
repo tidying for publication
</commit_message>
<xml_diff>
--- a/metadata/Extraction_Prep_Dates_Table.xlsx
+++ b/metadata/Extraction_Prep_Dates_Table.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10609"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10714"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lexikeene/Documents/Research/papers/github_copy/Old_Collections_Figures/metadata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A60602F-F369-C54D-91CC-2050308CF7FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE44338F-61F7-CD42-89E9-C439687F25C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1100" yWindow="940" windowWidth="28040" windowHeight="17200" xr2:uid="{BFA6B832-3A04-314D-A56A-7EC26A8902ED}"/>
   </bookViews>
@@ -47,12 +47,6 @@
     <t>Library Preparation Date</t>
   </si>
   <si>
-    <t>Secondary Library Preparation Date</t>
-  </si>
-  <si>
-    <t>Tertiary Library Preparation Date</t>
-  </si>
-  <si>
     <t>Albany1902_1 (now Albany_1908)</t>
   </si>
   <si>
@@ -195,6 +189,12 @@
   </si>
   <si>
     <t xml:space="preserve"> University of Guelph, The Centre for Biodiversity Genomics</t>
+  </si>
+  <si>
+    <t>Second Library Preparation Date</t>
+  </si>
+  <si>
+    <t>Third Library Preparation Date</t>
   </si>
 </sst>
 </file>
@@ -591,7 +591,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>1</v>
@@ -600,10 +600,10 @@
         <v>2</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>3</v>
+        <v>51</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>4</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
@@ -611,7 +611,7 @@
         <v>1004284</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C2" s="3">
         <v>44517</v>
@@ -620,18 +620,18 @@
         <v>44523</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C3" s="3">
         <v>44477</v>
@@ -640,10 +640,10 @@
         <v>44510</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
@@ -651,7 +651,7 @@
         <v>1004277</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C4" s="3">
         <v>44517</v>
@@ -671,7 +671,7 @@
         <v>1004279</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C5" s="3">
         <v>44517</v>
@@ -691,7 +691,7 @@
         <v>1004280</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C6" s="3">
         <v>44517</v>
@@ -700,10 +700,10 @@
         <v>44523</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
@@ -711,7 +711,7 @@
         <v>1004281</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C7" s="3">
         <v>44517</v>
@@ -731,7 +731,7 @@
         <v>1004282</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C8" s="3">
         <v>44517</v>
@@ -740,18 +740,18 @@
         <v>44523</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C9" s="3">
         <v>44386</v>
@@ -760,18 +760,18 @@
         <v>44515</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C10" s="3">
         <v>44477</v>
@@ -780,18 +780,18 @@
         <v>44515</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C11" s="3">
         <v>44477</v>
@@ -800,7 +800,7 @@
         <v>44510</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F11" s="3">
         <v>44753</v>
@@ -808,10 +808,10 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C12" s="3">
         <v>44477</v>
@@ -831,7 +831,7 @@
         <v>1004283</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C13" s="3">
         <v>44517</v>
@@ -840,10 +840,10 @@
         <v>44523</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
@@ -851,7 +851,7 @@
         <v>1004278</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C14" s="3">
         <v>44517</v>
@@ -868,10 +868,10 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C15" s="3">
         <v>44473</v>
@@ -880,18 +880,18 @@
         <v>44523</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C16" s="3">
         <v>44473</v>
@@ -900,18 +900,18 @@
         <v>44523</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C17" s="3">
         <v>44473</v>
@@ -920,18 +920,18 @@
         <v>44523</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C18" s="3">
         <v>44473</v>
@@ -940,18 +940,18 @@
         <v>44523</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C19" s="3">
         <v>44473</v>
@@ -960,18 +960,18 @@
         <v>44523</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C20" s="3">
         <v>44473</v>
@@ -988,10 +988,10 @@
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C21" s="3">
         <v>44486</v>
@@ -1000,18 +1000,18 @@
         <v>44515</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C22" s="3">
         <v>44486</v>
@@ -1028,10 +1028,10 @@
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C23" s="3">
         <v>44486</v>
@@ -1040,18 +1040,18 @@
         <v>44515</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C24" s="3">
         <v>44486</v>
@@ -1060,18 +1060,18 @@
         <v>44515</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C25" s="3">
         <v>44477</v>
@@ -1080,18 +1080,18 @@
         <v>44515</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C26" s="3">
         <v>44477</v>
@@ -1100,18 +1100,18 @@
         <v>44515</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C27" s="3">
         <v>44477</v>
@@ -1120,18 +1120,18 @@
         <v>44515</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C28" s="3">
         <v>44486</v>
@@ -1140,18 +1140,18 @@
         <v>44515</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C29" s="3">
         <v>44486</v>
@@ -1160,18 +1160,18 @@
         <v>44515</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C30" s="3">
         <v>44486</v>
@@ -1180,18 +1180,18 @@
         <v>44515</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C31" s="3">
         <v>44486</v>
@@ -1200,18 +1200,18 @@
         <v>44515</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C32" s="3">
         <v>44486</v>
@@ -1220,18 +1220,18 @@
         <v>44515</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F32" s="3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C33" s="3">
         <v>44477</v>
@@ -1240,18 +1240,18 @@
         <v>44515</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C34" s="3">
         <v>44477</v>
@@ -1260,18 +1260,18 @@
         <v>44515</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C35" s="3">
         <v>44477</v>
@@ -1280,18 +1280,18 @@
         <v>44515</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C36" s="3">
         <v>44435</v>
@@ -1308,10 +1308,10 @@
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C37" s="3">
         <v>44435</v>
@@ -1328,10 +1328,10 @@
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C38" s="3">
         <v>44473</v>
@@ -1340,18 +1340,18 @@
         <v>44523</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C39" s="3">
         <v>44473</v>
@@ -1360,18 +1360,18 @@
         <v>44523</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A40" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C40" s="3">
         <v>44473</v>
@@ -1388,10 +1388,10 @@
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C41" s="3">
         <v>44473</v>
@@ -1400,18 +1400,18 @@
         <v>44523</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C42" s="3">
         <v>44473</v>
@@ -1420,18 +1420,18 @@
         <v>44523</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F42" s="3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A43" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C43" s="3">
         <v>44473</v>
@@ -1440,18 +1440,18 @@
         <v>44523</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F43" s="3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C44" s="3">
         <v>44486</v>
@@ -1468,10 +1468,10 @@
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A45" s="1" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C45" s="3">
         <v>44486</v>
@@ -1488,10 +1488,10 @@
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C46" s="3">
         <v>44435</v>
@@ -1500,18 +1500,18 @@
         <v>44515</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F46" s="3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A47" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C47" s="3">
         <v>44435</v>
@@ -1520,7 +1520,7 @@
         <v>44515</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F47" s="3">
         <v>44753</v>

</xml_diff>